<commit_message>
Update application logic and data loaders for dashboard calculations
</commit_message>
<xml_diff>
--- a/Bom details.xlsx
+++ b/Bom details.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ngw11000658\Downloads\TEST\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ngw11000658\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E40CB479-F028-471C-BBAE-50AB50130014}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{97488B41-065E-42FD-878E-FCE738D11AA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{B3962CAF-7EBD-4156-AD70-194724843227}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,6 +34,9 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="2"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -1150,7 +1153,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1158,7 +1161,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -5414,39 +5417,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="0E2841"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="E8E8E8"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="156082"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="E97132"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="196B24"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="0F9ED5"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="A02B93"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="4EA72E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="467886"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -5479,9 +5482,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -5514,6 +5534,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -5575,13 +5612,6 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -5590,6 +5620,13 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -5654,18 +5691,38 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FE543E0-BCCA-4F7D-A8E9-5F3C1CA1C0DA}">
   <dimension ref="A1:E290"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>